<commit_message>
Atualização automática: Ranking CNB 2026
</commit_message>
<xml_diff>
--- a/Ranking_CNB_2026.xlsx
+++ b/Ranking_CNB_2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,26 @@
         <is>
           <t>Treinos</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Marcos Felix</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2,006,2 km</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>31.791 m</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>